<commit_message>
docs(changelog): extend merge changelog with post-6295d64 follow-up fixes
- 基线表 HEAD 更新至 c448b93（2026-09-09）
- 附录 Git 追溯补"6295d64 后收尾"行：4955a52 → c448b93 十个提交摘要
  （assets_box 重建 / 控件与捕获区恢复 / miniaudio UTF-8 DLL / Grid 菜单中文化 /
  Window id 对齐 / movement 重构 / 场景 uid 与面板参数 / extra window）
- xlsx 随行（同步工作区版本）
</commit_message>
<xml_diff>
--- a/ChangeReports/merge-changelog-1.4x-ec121415.xlsx
+++ b/ChangeReports/merge-changelog-1.4x-ec121415.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PNGTubeRemixWindowsPreV1.4.Build3\ForkRepos\GermanyShapy\PNGTuber-Remix-merge\ChangeReports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CB68C3E-1AF8-401E-B7A9-23AEAC23BEB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F6136A0-F220-4D6E-955B-9F91907B2E90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="11829" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -540,9 +540,6 @@
     <t>两侧均扩充 Global 信号与引用注册（Branch 大量信号、1.4.x 扩展），合成后信号链完整</t>
   </si>
   <si>
-    <t>Main/Scripts/Global.gd、main.gd、SpritesContainer.gd、SaveAndLoad.gd</t>
-  </si>
-  <si>
     <t>对象创建/删除/切换状态/显隐等跨系统信号全部正常触发（重点 regression）</t>
   </si>
   <si>
@@ -555,9 +552,6 @@
     <t>Skew 平铺 Layouts、控件 connection 直连为手工合成结果</t>
   </si>
   <si>
-    <t>UI/EditorUI/RightUI/Components/properties.tscn、model_effects.tscn、properties_script.gd、model_effects.gd</t>
-  </si>
-  <si>
     <t>属性页所有滑条/输入框/按钮可操作且写回正确；特效页参数联动</t>
   </si>
   <si>
@@ -585,9 +579,6 @@
     <t>1.4.x 基线 + 插入 Branch 自定义热键区块（HotkeyItemList）</t>
   </si>
   <si>
-    <t>UI/EditorUI/TopUI/Components/Settings_popup.tscn、hotkey_item.tscn、settings_script.gd</t>
-  </si>
-  <si>
     <t>设置页除热键外其余项（检测/音频/画质/快捷键总开关）无回归；热键区块完整可用</t>
   </si>
   <si>
@@ -597,12 +588,6 @@
     <t>movement/animation_tab 裁决提示</t>
   </si>
   <si>
-    <t>取 1.4.x 版：Branch 在此处语义改动（含部分跳跃/物理语义）未进入合流产物，以 1.4.x 行为为准</t>
-  </si>
-  <si>
-    <t>UI/EditorUI/RightUI/Components/movement.tscn、animation_tab.tscn、movement_tab.gd、animation_tab.gd</t>
-  </si>
-  <si>
     <t>① Branch(4.4) 老用户如有依赖旧 movement 行为的场景请复核提报；② 1.4.x 用户按原行为回归</t>
   </si>
   <si>
@@ -615,9 +600,6 @@
     <t>reaction_config.gd、global_calculations.gd 两侧均改；wiggly_appendage_2d.gd 双方优化合成</t>
   </si>
   <si>
-    <t>Scripts/Objects/ObjectComponents/reaction_config.gd、Scripts/Global/global_calculations.gd、addons/wiggly_appendage_2d/wiggly_appendage_2d.gd、layers_panel_scripts.gd</t>
-  </si>
-  <si>
     <t>反应(表情/音频)触发、层级面板联动、附件跟随三项冒烟</t>
   </si>
   <si>
@@ -643,9 +625,6 @@
   </si>
   <si>
     <t>main.tscn 直跑噪音清理</t>
-  </si>
-  <si>
-    <t>清理 4 个上游遗留失效 UI 引用（light_source UI 路径等），根治启动 SCRIPT ERROR 噪音（4.4 侧同步提交 1bee220）</t>
   </si>
   <si>
     <t>a3077ac（对应 7abf312/1bee220）</t>
@@ -1027,6 +1006,34 @@
       </rPr>
       <t>Settings_popup 1.4.x 基线+Branch 热键区块；assets_box 整文件取 Branch；Global.gd/sprite_object.gd 缩进损坏修复；assets_box CheckBox changed→toggled 无效连接修复</t>
     </r>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Main/Scripts/Global.gd、main.gd、SpritesContainer.gd、SaveAndLoad.gd</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>UI/EditorUI/RightUI/Components/properties.tscn、model_effects.tscn、properties_script.gd、model_effects.gd</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>UI/EditorUI/TopUI/Components/Settings_popup.tscn、hotkey_item.tscn、settings_script.gd</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>取 1.4.x 版：Branch 在此处语义改动（含部分跳跃/物理语义）未进入合流产物，以 1.4.x 行为为准</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>UI/EditorUI/RightUI/Components/movement.tscn、animation_tab.tscn、movement_tab.gd、animation_tab.gd</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Scripts/Objects/ObjectComponents/reaction_config.gd、Scripts/Global/global_calculations.gd、addons/wiggly_appendage_2d/wiggly_appendage_2d.gd、layers_panel_scripts.gd</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>清理 4 个上游遗留失效 UI 引用（light_source UI 路径等），根治启动 SCRIPT ERROR 噪音（4.4 侧同步提交 1bee220）</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -1047,12 +1054,14 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
     </font>
     <font>
@@ -1071,7 +1080,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1109,6 +1118,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -1137,7 +1158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1170,6 +1191,21 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2126,14 +2162,14 @@
       </c>
     </row>
     <row r="33" spans="1:6" ht="70.75" x14ac:dyDescent="0.3">
-      <c r="A33" s="2" t="s">
+      <c r="A33" s="13" t="s">
         <v>163</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="B33" s="12" t="s">
         <v>164</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>329</v>
+        <v>322</v>
       </c>
       <c r="D33" s="3" t="s">
         <v>165</v>
@@ -2146,283 +2182,283 @@
       </c>
     </row>
     <row r="34" spans="1:6" ht="28.3" x14ac:dyDescent="0.3">
-      <c r="A34" s="2" t="s">
+      <c r="A34" s="13" t="s">
         <v>168</v>
       </c>
-      <c r="B34" s="3" t="s">
+      <c r="B34" s="12" t="s">
         <v>169</v>
       </c>
-      <c r="C34" s="3" t="s">
+      <c r="C34" s="12" t="s">
         <v>170</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>171</v>
+        <v>323</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>166</v>
       </c>
       <c r="F34" s="3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="42.45" x14ac:dyDescent="0.3">
+      <c r="A35" s="13" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" ht="42.45" x14ac:dyDescent="0.3">
-      <c r="A35" s="2" t="s">
+      <c r="B35" s="12" t="s">
         <v>173</v>
       </c>
-      <c r="B35" s="3" t="s">
+      <c r="C35" s="12" t="s">
         <v>174</v>
       </c>
-      <c r="C35" s="3" t="s">
-        <v>175</v>
-      </c>
       <c r="D35" s="3" t="s">
-        <v>176</v>
+        <v>324</v>
       </c>
       <c r="E35" s="6" t="s">
         <v>166</v>
       </c>
       <c r="F35" s="3" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="28.3" x14ac:dyDescent="0.3">
+      <c r="A36" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="B36" s="15" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" ht="28.3" x14ac:dyDescent="0.3">
-      <c r="A36" s="2" t="s">
+      <c r="C36" s="12" t="s">
         <v>178</v>
       </c>
-      <c r="B36" s="3" t="s">
+      <c r="D36" s="3" t="s">
         <v>179</v>
-      </c>
-      <c r="C36" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="D36" s="3" t="s">
-        <v>181</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>166</v>
       </c>
       <c r="F36" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="28.3" x14ac:dyDescent="0.3">
+      <c r="A37" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="B37" s="12" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" ht="28.3" x14ac:dyDescent="0.3">
-      <c r="A37" s="2" t="s">
+      <c r="C37" s="12" t="s">
         <v>183</v>
       </c>
-      <c r="B37" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="C37" s="3" t="s">
-        <v>185</v>
-      </c>
       <c r="D37" s="3" t="s">
-        <v>186</v>
+        <v>325</v>
       </c>
       <c r="E37" s="6" t="s">
         <v>166</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="42.45" x14ac:dyDescent="0.3">
-      <c r="A38" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="C38" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="D38" s="3" t="s">
-        <v>191</v>
+      <c r="A38" s="13" t="s">
+        <v>185</v>
+      </c>
+      <c r="B38" s="12" t="s">
+        <v>186</v>
+      </c>
+      <c r="C38" s="12" t="s">
+        <v>326</v>
+      </c>
+      <c r="D38" s="16" t="s">
+        <v>327</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>166</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="56.6" x14ac:dyDescent="0.3">
-      <c r="A39" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="C39" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="D39" s="3" t="s">
-        <v>196</v>
+      <c r="A39" s="13" t="s">
+        <v>188</v>
+      </c>
+      <c r="B39" s="12" t="s">
+        <v>189</v>
+      </c>
+      <c r="C39" s="12" t="s">
+        <v>190</v>
+      </c>
+      <c r="D39" s="16" t="s">
+        <v>328</v>
       </c>
       <c r="E39" s="6" t="s">
         <v>166</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="28.3" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="42.45" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>206</v>
+        <v>329</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="E41" s="7" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="42.45" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="E42" s="7" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="28.3" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="E43" s="7" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="E44" s="7" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="28.3" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="E45" s="7" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="42.45" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="E46" s="7" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="28.3" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="E47" s="7" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
     </row>
   </sheetData>
@@ -2443,114 +2479,114 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="28.3" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="28.3" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="28.3" x14ac:dyDescent="0.3">
       <c r="A13" s="9" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="28.3" x14ac:dyDescent="0.3">
       <c r="A14" s="9" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
     </row>
   </sheetData>
@@ -2570,79 +2606,79 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="70.75" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="28.3" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
-        <v>273</v>
+        <v>266</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="42.45" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>278</v>
+        <v>271</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="113.15" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>280</v>
+        <v>273</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>281</v>
+        <v>274</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="99" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>282</v>
+        <v>275</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="28.3" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>285</v>
+        <v>278</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>286</v>
+        <v>279</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -2652,107 +2688,107 @@
     </row>
     <row r="9" spans="1:3" ht="28.3" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
-        <v>287</v>
+        <v>280</v>
       </c>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>289</v>
+        <v>282</v>
       </c>
       <c r="C10" s="10"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
-        <v>290</v>
+        <v>283</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>291</v>
+        <v>284</v>
       </c>
       <c r="C11" s="10"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="C12" s="10"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="9" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>295</v>
+        <v>288</v>
       </c>
       <c r="C13" s="10"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="9" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>297</v>
+        <v>290</v>
       </c>
       <c r="C14" s="10"/>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="9" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="C15" s="10"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="9" t="s">
-        <v>300</v>
+        <v>293</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
       <c r="C16" s="10"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="9" t="s">
-        <v>302</v>
+        <v>295</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>303</v>
+        <v>296</v>
       </c>
       <c r="C17" s="10"/>
     </row>
     <row r="18" spans="1:3" ht="28.3" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
-        <v>304</v>
+        <v>297</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>305</v>
+        <v>298</v>
       </c>
       <c r="C18" s="10"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="s">
-        <v>306</v>
+        <v>299</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>307</v>
+        <v>300</v>
       </c>
       <c r="C19" s="10"/>
     </row>
     <row r="20" spans="1:3" ht="28.3" x14ac:dyDescent="0.3">
       <c r="A20" s="9" t="s">
-        <v>308</v>
+        <v>301</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="C20" s="10"/>
     </row>
@@ -2763,89 +2799,89 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="9" t="s">
-        <v>310</v>
+        <v>303</v>
       </c>
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
     </row>
     <row r="23" spans="1:3" ht="56.6" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>312</v>
+        <v>305</v>
       </c>
       <c r="C23" s="10"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="9" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="C24" s="10"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="9" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>316</v>
+        <v>309</v>
       </c>
       <c r="C25" s="10"/>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="9" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>318</v>
+        <v>311</v>
       </c>
       <c r="C26" s="10"/>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="s">
-        <v>319</v>
+        <v>312</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="C27" s="10"/>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="9" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>322</v>
+        <v>315</v>
       </c>
       <c r="C28" s="10"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" s="9" t="s">
-        <v>323</v>
+        <v>316</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>324</v>
+        <v>317</v>
       </c>
       <c r="C29" s="10"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" s="9" t="s">
-        <v>325</v>
+        <v>318</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
       <c r="C30" s="10"/>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" s="9" t="s">
-        <v>327</v>
+        <v>320</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>328</v>
+        <v>321</v>
       </c>
       <c r="C31" s="10"/>
     </row>

</xml_diff>